<commit_message>
Add extent time series table and update all examples
New in extent accounts:
- Extent Time Series sheet in template (track across multiple periods,
  auto-calculates total change and net change per period)
- Extent Time Series sheet in examples (4 periods: 2010, 2014, 2018,
  2023 showing coral/seagrass declining, mangroves increasing)
- Net change per period sub-table showing trends over time

Updated HTML examples slide with time series table and interpretation
box explaining what the trajectory reveals that a single snapshot cannot.

The extent template now has 4 sheets:
1. Extent Account (single period opening/closing)
2. Extent Time Series (multi-period, builds over time)
3. Change Matrix (cross-tabulation)
4. Instructions

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/s-s-event-bogor/sessions/day-2/clinic/examples/example_completed_accounts.xlsx
+++ b/s-s-event-bogor/sessions/day-2/clinic/examples/example_completed_accounts.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extent Account" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Matrix" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Condition Account" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services - Part A Physical" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services - Part B Monetary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extent Time Series" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Matrix" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Condition Account" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services - Part A Physical" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services - Part B Monetary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,10 +22,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="+0.00;-0.00;0.00"/>
-    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
-    <numFmt numFmtId="166" formatCode="+0.00;-0.00"/>
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="+#,##0;-#,##0"/>
+    <numFmt numFmtId="167" formatCode="+0.00;-0.00;0.00"/>
+    <numFmt numFmtId="168" formatCode="+0.00;-0.00"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -127,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -144,11 +147,21 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -156,7 +169,7 @@
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -164,17 +177,13 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -860,6 +869,344 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="003B9C7B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Table 1b: Ecosystem Extent Time Series</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Coastal District Example, 2010 to 2023 (multiple accounting periods)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Each period's closing extent becomes the next period's opening extent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Ecosystem type</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>2010
+(ha)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>2014
+(ha)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>2018
+(ha)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>2023
+(ha)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Total change
+2010-2023
+(ha)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Total change
+(%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Coral reefs (M1.3)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>1420</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>1340</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>1240</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>1180</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>-240</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>-0.169</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Seagrass (M1.1)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>950</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>910</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>860</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>825</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>-125</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>-0.132</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mangroves (MFT1.2)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>280</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>290</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>315</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>340</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>0.214</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>7350</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>7460</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>7585</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>7655</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>305</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>0.04099999999999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Total accounting area</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>10000</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Net change per accounting period</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Ecosystem type</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>2010-2014
+(ha)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>2014-2018
+(ha)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>2018-2023
+(ha)</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Trend</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Coral reefs</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>-80</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>-100</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>-60</v>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Declining (slowing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Seagrass</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>-40</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>-50</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>-35</v>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Declining (slowing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Mangroves</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Increasing (stable rate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Trend interpretation: compare magnitude of net change across periods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Coral and seagrass losses are slowing, suggesting either reduced pressures or approaching a floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Mangrove gains are consistent, likely reflecting sustained restoration programmes.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="000A5455"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -928,7 +1275,7 @@
           <t>Coral reefs</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="13" t="n">
         <v>1140</v>
       </c>
       <c r="C5" s="6" t="n">
@@ -953,7 +1300,7 @@
       <c r="B6" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="13" t="n">
         <v>790</v>
       </c>
       <c r="D6" s="6" t="n">
@@ -978,7 +1325,7 @@
       <c r="C7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="13" t="n">
         <v>300</v>
       </c>
       <c r="E7" s="6" t="n">
@@ -1003,7 +1350,7 @@
       <c r="D8" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="13" t="n">
         <v>7500</v>
       </c>
       <c r="F8" s="6" t="n">
@@ -1044,7 +1391,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="003B9C7B"/>
@@ -1146,12 +1493,12 @@
           <t>Live coral cover</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>Higher is better</t>
         </is>
@@ -1159,22 +1506,22 @@
       <c r="D5" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="14" t="n">
         <v>31.13</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="15" t="n">
         <v>0.62</v>
       </c>
-      <c r="G5" s="10" t="n">
+      <c r="G5" s="14" t="n">
         <v>26.63</v>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="H5" s="15" t="n">
         <v>0.53</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="I5" s="16" t="n">
         <v>-0.09</v>
       </c>
-      <c r="J5" s="9" t="inlineStr">
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -1186,12 +1533,12 @@
           <t>Fleshy macroalgae cover</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>Higher is worse</t>
         </is>
@@ -1199,22 +1546,22 @@
       <c r="D6" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="E6" s="14" t="n">
         <v>22.63</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="15" t="n">
         <v>0.62</v>
       </c>
-      <c r="G6" s="10" t="n">
+      <c r="G6" s="14" t="n">
         <v>27.38</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="H6" s="15" t="n">
         <v>0.54</v>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="16" t="n">
         <v>-0.08</v>
       </c>
-      <c r="J6" s="9" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -1226,12 +1573,12 @@
           <t>Fish biomass</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>kg/ha</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Higher is better</t>
         </is>
@@ -1239,22 +1586,22 @@
       <c r="D7" s="6" t="n">
         <v>500</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="14" t="n">
         <v>213.75</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="F7" s="15" t="n">
         <v>0.43</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="14" t="n">
         <v>193.75</v>
       </c>
-      <c r="H7" s="11" t="n">
+      <c r="H7" s="15" t="n">
         <v>0.39</v>
       </c>
-      <c r="I7" s="12" t="n">
+      <c r="I7" s="16" t="n">
         <v>-0.04</v>
       </c>
-      <c r="J7" s="9" t="inlineStr">
+      <c r="J7" s="12" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -1266,12 +1613,12 @@
           <t>Coral recruit density</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>per m2</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Higher is better</t>
         </is>
@@ -1279,22 +1626,22 @@
       <c r="D8" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="14" t="n">
         <v>8.5</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="15" t="n">
         <v>0.57</v>
       </c>
-      <c r="G8" s="10" t="n">
+      <c r="G8" s="14" t="n">
         <v>6.2</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="H8" s="15" t="n">
         <v>0.41</v>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="I8" s="16" t="n">
         <v>-0.15</v>
       </c>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -1306,12 +1653,12 @@
           <t>Reef relief</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>cm</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Higher is better</t>
         </is>
@@ -1319,22 +1666,22 @@
       <c r="D9" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="14" t="n">
         <v>82.5</v>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="F9" s="15" t="n">
         <v>0.55</v>
       </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="14" t="n">
         <v>78</v>
       </c>
-      <c r="H9" s="11" t="n">
+      <c r="H9" s="15" t="n">
         <v>0.52</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="I9" s="16" t="n">
         <v>-0.03</v>
       </c>
-      <c r="J9" s="9" t="inlineStr">
+      <c r="J9" s="12" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
@@ -1346,12 +1693,12 @@
           <t>Bleaching prevalence</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>% colonies</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>Higher is worse</t>
         </is>
@@ -1359,22 +1706,22 @@
       <c r="D10" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="14" t="n">
         <v>8.5</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="15" t="n">
         <v>0.92</v>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="G10" s="14" t="n">
         <v>18.3</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="15" t="n">
         <v>0.82</v>
       </c>
-      <c r="I10" s="12" t="n">
+      <c r="I10" s="16" t="n">
         <v>-0.1</v>
       </c>
-      <c r="J10" s="9" t="inlineStr">
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -1386,25 +1733,25 @@
           <t>Composite Condition Index</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>average</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="14" t="n"/>
-      <c r="E11" s="14" t="n"/>
-      <c r="F11" s="15" t="n">
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+      <c r="E11" s="18" t="n"/>
+      <c r="F11" s="19" t="n">
         <v>0.62</v>
       </c>
-      <c r="G11" s="14" t="n"/>
-      <c r="H11" s="15" t="n">
+      <c r="G11" s="18" t="n"/>
+      <c r="H11" s="19" t="n">
         <v>0.53</v>
       </c>
-      <c r="I11" s="16" t="n">
+      <c r="I11" s="20" t="n">
         <v>-0.08</v>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="21" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -1429,7 +1776,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="003B9C7B"/>
@@ -1507,12 +1854,12 @@
           <t>Wild fish provisioning</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Provisioning</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>kg/yr</t>
         </is>
@@ -1536,12 +1883,12 @@
           <t>Wood provisioning</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Provisioning</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>tonnes/yr</t>
         </is>
@@ -1561,12 +1908,12 @@
           <t>Carbon sequestration</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Regulating</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Mg CO2/yr</t>
         </is>
@@ -1588,12 +1935,12 @@
           <t>Coastal protection</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Regulating</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>m coastline</t>
         </is>
@@ -1615,12 +1962,12 @@
           <t>Nursery habitat</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Regulating</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>kg biomass/yr</t>
         </is>
@@ -1642,12 +1989,12 @@
           <t>Sediment retention</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Regulating</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>m3 CaCO3/yr</t>
         </is>
@@ -1667,12 +2014,12 @@
           <t>Recreation (reef diving)</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Cultural</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>visitors/yr</t>
         </is>
@@ -1692,12 +2039,12 @@
           <t>Recreation (mangrove tours)</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Cultural</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>trips/yr</t>
         </is>
@@ -1717,12 +2064,12 @@
           <t>Gleaning</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Cultural</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>hours/yr</t>
         </is>
@@ -1742,12 +2089,12 @@
           <t>Gleaning harvest</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Cultural</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>kg/yr</t>
         </is>
@@ -1773,7 +2120,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="000A5455"/>
@@ -1852,12 +2199,12 @@
           <t>Wild fish provisioning</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Resource rent</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
@@ -1881,12 +2228,12 @@
           <t>Wood provisioning</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Substitute cost</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>Non-market</t>
         </is>
@@ -1906,12 +2253,12 @@
           <t>Carbon sequestration</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Social cost of carbon</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Non-market</t>
         </is>
@@ -1933,12 +2280,12 @@
           <t>Coastal protection</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Replacement cost</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Non-market</t>
         </is>
@@ -1960,12 +2307,12 @@
           <t>Nursery habitat</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Productivity change</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Market (indirect)</t>
         </is>
@@ -1987,12 +2334,12 @@
           <t>Sediment retention</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Replacement cost</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>Non-market</t>
         </is>
@@ -2012,12 +2359,12 @@
           <t>Recreation (reef)</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Direct expenditure</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
@@ -2037,12 +2384,12 @@
           <t>Recreation (mangrove)</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Direct expenditure</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
@@ -2062,12 +2409,12 @@
           <t>Gleaning</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Equivalent wage</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
@@ -2087,8 +2434,8 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="14" t="n"/>
+      <c r="B14" s="18" t="n"/>
+      <c r="C14" s="18" t="n"/>
       <c r="D14" s="5" t="n">
         <v>3113750</v>
       </c>
@@ -2128,7 +2475,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="003B9C7B"/>
@@ -2160,7 +2507,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Extent (Table 1)</t>
         </is>
@@ -2208,7 +2555,7 @@
       <c r="D6" s="6" t="n">
         <v>-60</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="8" t="n">
         <v>-0.048</v>
       </c>
     </row>
@@ -2227,7 +2574,7 @@
       <c r="D7" s="6" t="n">
         <v>-35</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="8" t="n">
         <v>-0.04099999999999999</v>
       </c>
     </row>
@@ -2246,12 +2593,12 @@
       <c r="D8" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="8" t="n">
         <v>0.079</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Condition (Table 3)</t>
         </is>
@@ -2290,16 +2637,16 @@
           <t>Live coral cover</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="15" t="n">
         <v>0.62</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="15" t="n">
         <v>0.53</v>
       </c>
-      <c r="D12" s="20" t="n">
+      <c r="D12" s="22" t="n">
         <v>-0.09</v>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -2311,16 +2658,16 @@
           <t>Macroalgae cover</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="15" t="n">
         <v>0.62</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="15" t="n">
         <v>0.54</v>
       </c>
-      <c r="D13" s="20" t="n">
+      <c r="D13" s="22" t="n">
         <v>-0.08</v>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -2332,16 +2679,16 @@
           <t>Fish biomass</t>
         </is>
       </c>
-      <c r="B14" s="11" t="n">
+      <c r="B14" s="15" t="n">
         <v>0.43</v>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="15" t="n">
         <v>0.39</v>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D14" s="22" t="n">
         <v>-0.04</v>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -2353,23 +2700,23 @@
           <t>Composite</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n">
+      <c r="B15" s="15" t="n">
         <v>0.62</v>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="15" t="n">
         <v>0.53</v>
       </c>
-      <c r="D15" s="20" t="n">
+      <c r="D15" s="22" t="n">
         <v>-0.08</v>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>Ecosystem Services (Tables 4a + 4b)</t>
         </is>
@@ -2404,7 +2751,7 @@
           <t>Fish provisioning</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>180,000 kg/yr</t>
         </is>
@@ -2412,7 +2759,7 @@
       <c r="C20" s="6" t="n">
         <v>210000</v>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>Resource rent</t>
         </is>
@@ -2424,7 +2771,7 @@
           <t>Carbon sequestration</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>2,335 Mg CO2/yr</t>
         </is>
@@ -2432,7 +2779,7 @@
       <c r="C21" s="6" t="n">
         <v>119085</v>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>SCC</t>
         </is>
@@ -2444,7 +2791,7 @@
           <t>Coastal protection</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>15,500 m coastline</t>
         </is>
@@ -2452,7 +2799,7 @@
       <c r="C22" s="6" t="n">
         <v>1375000</v>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D22" s="12" t="inlineStr">
         <is>
           <t>Replacement cost</t>
         </is>
@@ -2464,7 +2811,7 @@
           <t>Nursery habitat</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>7,300 kg biomass/yr</t>
         </is>
@@ -2472,7 +2819,7 @@
       <c r="C23" s="6" t="n">
         <v>127750</v>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Productivity change</t>
         </is>
@@ -2484,7 +2831,7 @@
           <t>Sediment retention</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>8,400 m3/yr</t>
         </is>
@@ -2492,7 +2839,7 @@
       <c r="C24" s="6" t="n">
         <v>420000</v>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Replacement cost</t>
         </is>
@@ -2504,7 +2851,7 @@
           <t>Recreation</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>17,400 visitors/yr</t>
         </is>
@@ -2512,7 +2859,7 @@
       <c r="C25" s="6" t="n">
         <v>1359000</v>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>Direct expenditure</t>
         </is>
@@ -2524,7 +2871,7 @@
           <t>Gleaning</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>18,000 hours/yr</t>
         </is>
@@ -2532,7 +2879,7 @@
       <c r="C26" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>Equivalent wage</t>
         </is>
@@ -2544,7 +2891,7 @@
           <t>Wood provisioning</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>85 tonnes/yr</t>
         </is>
@@ -2552,7 +2899,7 @@
       <c r="C27" s="6" t="n">
         <v>12750</v>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Substitute cost</t>
         </is>
@@ -2564,11 +2911,11 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr"/>
+      <c r="B28" s="12" t="inlineStr"/>
       <c r="C28" s="5" t="n">
         <v>3686585</v>
       </c>
-      <c r="D28" s="9" t="inlineStr"/>
+      <c r="D28" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add data sources reference for all ecosystem service calculations
New file: services/data-sources-by-service.md
- Comprehensive data source guide for all 7 services
- Organized by Part A (physical) and Part B (monetary)
- Includes specific URLs, dataset names, and Tier 1 shortcuts
- NCP rate table with conservative/central/high estimates and sources
- Carbon price comparison table (SCC, EU ETS, voluntary, VCS)
- Quick reference: 14 global open datasets with URLs

New sheet in example_completed_accounts.xlsx: "Data Sources"
- Full lookup table: service, data needed, Part A/B, source, URL
- Global open datasets section at bottom
- GOAP-styled formatting

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/s-s-event-bogor/sessions/day-2/clinic/examples/example_completed_accounts.xlsx
+++ b/s-s-event-bogor/sessions/day-2/clinic/examples/example_completed_accounts.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services - Part A Physical" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services - Part B Monetary" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Sources" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
     <numFmt numFmtId="167" formatCode="+0.00;-0.00;0.00"/>
     <numFmt numFmtId="168" formatCode="+0.00;-0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,6 +77,11 @@
       <b val="1"/>
       <color rgb="000A5455"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="005EB593"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -130,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -186,6 +192,11 @@
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2920,4 +2931,1110 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="003B9C7B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Data Sources for Ecosystem Service Calculations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Where to find the data for each service (Part A physical and Part B monetary)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>SERVICE</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>DATA NEEDED</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>PART</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>URL / REFERENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>Fish provisioning</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Total catch (kg/yr)</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>National fisheries agency landing records</t>
+        </is>
+      </c>
+      <c r="E5" s="25" t="inlineStr">
+        <is>
+          <t>FAO: fao.org/fishery</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>Fish provisioning</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Catch by species</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>Landing site surveys, fisher cooperatives</t>
+        </is>
+      </c>
+      <c r="E6" s="25" t="inlineStr">
+        <is>
+          <t>FishBase: fishbase.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>Fish provisioning</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Catch by country (Tier 1)</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>FAO FishStatJ or Sea Around Us</t>
+        </is>
+      </c>
+      <c r="E7" s="25" t="inlineStr">
+        <is>
+          <t>seaaroundus.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>Fish provisioning</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Market prices (USD/kg)</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>Local fish market surveys, national stats</t>
+        </is>
+      </c>
+      <c r="E8" s="25" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>Fish provisioning</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Fishing costs</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>Fisher household surveys</t>
+        </is>
+      </c>
+      <c r="E9" s="25" t="inlineStr">
+        <is>
+          <t>GOAP survey templates</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>Carbon sequestration</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Ecosystem extent (ha)</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>Extent account, or global datasets</t>
+        </is>
+      </c>
+      <c r="E11" s="25" t="inlineStr">
+        <is>
+          <t>globalmangrovewatch.org, allencoralatlas.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>Carbon sequestration</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>NCP rates (Mg CO2/ha/yr)</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>Published literature</t>
+        </is>
+      </c>
+      <c r="E12" s="25" t="inlineStr">
+        <is>
+          <t>Alongi (2014), Fourqurean et al. (2012)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>Carbon sequestration</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>IPCC default rates</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>IPCC Wetlands Supplement (2013)</t>
+        </is>
+      </c>
+      <c r="E13" s="25" t="inlineStr">
+        <is>
+          <t>ipcc.ch</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>Carbon sequestration</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Primary carbon data (Tier 2-3)</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>Field: soil cores, allometric equations</t>
+        </is>
+      </c>
+      <c r="E14" s="25" t="inlineStr">
+        <is>
+          <t>National forest inventories</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>Carbon sequestration</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Social cost of carbon</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>US EPA Interagency Working Group</t>
+        </is>
+      </c>
+      <c r="E15" s="25" t="inlineStr">
+        <is>
+          <t>USD 51/Mg CO2 (2021 central)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>Carbon sequestration</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Voluntary market price</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Ecosystem Marketplace</t>
+        </is>
+      </c>
+      <c r="E16" s="25" t="inlineStr">
+        <is>
+          <t>ecosystemmarketplace.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>Carbon sequestration</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>VCS blue carbon credits</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Verra project registry</t>
+        </is>
+      </c>
+      <c r="E17" s="25" t="inlineStr">
+        <is>
+          <t>verra.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>Coastal protection</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Ecosystem extent along coast</t>
+        </is>
+      </c>
+      <c r="C19" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>GIS overlay of extent map + coastline</t>
+        </is>
+      </c>
+      <c r="E19" s="25" t="inlineStr">
+        <is>
+          <t>From extent account</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>Coastal protection</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Buildings behind buffer</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>OpenStreetMap, national cadastres</t>
+        </is>
+      </c>
+      <c r="E20" s="25" t="inlineStr">
+        <is>
+          <t>openstreetmap.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>Coastal protection</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Population behind buffer</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>Census data, WorldPop</t>
+        </is>
+      </c>
+      <c r="E21" s="25" t="inlineStr">
+        <is>
+          <t>worldpop.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>Coastal protection</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>Seawall cost (USD/m)</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>Engineering firms, govt infrastructure budgets</t>
+        </is>
+      </c>
+      <c r="E22" s="25" t="inlineStr">
+        <is>
+          <t>Range: USD 2,000-15,000/m</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>Coastal protection</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>Wave attenuation data (Tier 3)</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>Wave models, buoy data</t>
+        </is>
+      </c>
+      <c r="E23" s="25" t="inlineStr">
+        <is>
+          <t>NOAA WaveWatch III</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>Nursery habitat</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Fish density (nursery vs non-nursery)</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>Field surveys (UVC, seine nets)</t>
+        </is>
+      </c>
+      <c r="E25" s="25" t="inlineStr">
+        <is>
+          <t>National monitoring programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>Nursery habitat</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>Log Response Ratio (LRR)</t>
+        </is>
+      </c>
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>Literature meta-analyses</t>
+        </is>
+      </c>
+      <c r="E26" s="25" t="inlineStr">
+        <is>
+          <t>Coral: 31%, Seagrass: 13%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>Nursery habitat</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>Total fish biomass</t>
+        </is>
+      </c>
+      <c r="C27" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>From fish provisioning account</t>
+        </is>
+      </c>
+      <c r="E27" s="25" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>Nursery habitat</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Market price of fish</t>
+        </is>
+      </c>
+      <c r="C28" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>Same as fish provisioning</t>
+        </is>
+      </c>
+      <c r="E28" s="25" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>Visitor arrivals</t>
+        </is>
+      </c>
+      <c r="C30" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>National tourism authority, UNWTO</t>
+        </is>
+      </c>
+      <c r="E30" s="25" t="inlineStr">
+        <is>
+          <t>unwto.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>Dive/snorkel activity</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>Dive centres, tour operators</t>
+        </is>
+      </c>
+      <c r="E31" s="25" t="inlineStr">
+        <is>
+          <t>PADI statistics, local associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="23" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>MPA visitor counts</t>
+        </is>
+      </c>
+      <c r="C32" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>Park management, entry permits</t>
+        </is>
+      </c>
+      <c r="E32" s="25" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>Activity fees</t>
+        </is>
+      </c>
+      <c r="C33" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>Operator records, online pricing</t>
+        </is>
+      </c>
+      <c r="E33" s="25" t="inlineStr">
+        <is>
+          <t>Direct observation</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="23" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>Visitor expenditure surveys</t>
+        </is>
+      </c>
+      <c r="C34" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>Tourist surveys, accommodation records</t>
+        </is>
+      </c>
+      <c r="E34" s="25" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="23" t="inlineStr">
+        <is>
+          <t>Gleaning</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>Gleaner counts and effort</t>
+        </is>
+      </c>
+      <c r="C36" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>Household surveys, community monitoring</t>
+        </is>
+      </c>
+      <c r="E36" s="25" t="inlineStr">
+        <is>
+          <t>Participatory methods</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="23" t="inlineStr">
+        <is>
+          <t>Gleaning</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>Harvest by species (kg)</t>
+        </is>
+      </c>
+      <c r="C37" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>Gleaner interviews, landing measurements</t>
+        </is>
+      </c>
+      <c r="E37" s="25" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr">
+        <is>
+          <t>Gleaning</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>Local wage rate</t>
+        </is>
+      </c>
+      <c r="C38" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>National statistics, minimum wage</t>
+        </is>
+      </c>
+      <c r="E38" s="25" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t>Gleaning</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>Market prices for harvest</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>Local market surveys</t>
+        </is>
+      </c>
+      <c r="E39" s="25" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="23" t="inlineStr">
+        <is>
+          <t>Sediment retention</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>CaCO3 production rates</t>
+        </is>
+      </c>
+      <c r="C41" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>Literature</t>
+        </is>
+      </c>
+      <c r="E41" s="25" t="inlineStr">
+        <is>
+          <t>Perry et al. (2012)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="23" t="inlineStr">
+        <is>
+          <t>Sediment retention</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="inlineStr">
+        <is>
+          <t>Beach nourishment cost</t>
+        </is>
+      </c>
+      <c r="C42" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
+        <is>
+          <t>Coastal management agencies</t>
+        </is>
+      </c>
+      <c r="E42" s="25" t="inlineStr">
+        <is>
+          <t>Range: USD 5-20/m3</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>Global Open Datasets (free, get started quickly)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>What it provides</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Allen Coral Atlas</t>
+        </is>
+      </c>
+      <c r="B46" s="25" t="inlineStr">
+        <is>
+          <t>allencoralatlas.org</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>Coral reef and seagrass extent, benthic cover</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Global Mangrove Watch</t>
+        </is>
+      </c>
+      <c r="B47" s="25" t="inlineStr">
+        <is>
+          <t>globalmangrovewatch.org</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>Mangrove extent 1996-2020, canopy height, biomass</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Global Fishing Watch</t>
+        </is>
+      </c>
+      <c r="B48" s="25" t="inlineStr">
+        <is>
+          <t>globalfishingwatch.org</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>Fishing effort, vessel tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Sea Around Us</t>
+        </is>
+      </c>
+      <c r="B49" s="25" t="inlineStr">
+        <is>
+          <t>seaaroundus.org</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>Reconstructed catch by country, EEZ, species</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>FAO FishStatJ</t>
+        </is>
+      </c>
+      <c r="B50" s="25" t="inlineStr">
+        <is>
+          <t>fao.org/fishery/statistics</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>National fisheries production and trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>UNWTO</t>
+        </is>
+      </c>
+      <c r="B51" s="25" t="inlineStr">
+        <is>
+          <t>unwto.org</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="inlineStr">
+        <is>
+          <t>International tourism arrivals and receipts</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>WorldPop</t>
+        </is>
+      </c>
+      <c r="B52" s="25" t="inlineStr">
+        <is>
+          <t>worldpop.org</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>Gridded population estimates</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="B53" s="25" t="inlineStr">
+        <is>
+          <t>openstreetmap.org</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>Building footprints, infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>NOAA Coral Reef Watch</t>
+        </is>
+      </c>
+      <c r="B54" s="25" t="inlineStr">
+        <is>
+          <t>coralreefwatch.noaa.gov</t>
+        </is>
+      </c>
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>SST, DHW, bleaching alerts</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>ESVD</t>
+        </is>
+      </c>
+      <c r="B55" s="25" t="inlineStr">
+        <is>
+          <t>esvd.info</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="inlineStr">
+        <is>
+          <t>Published valuations for value transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Ecosystem Marketplace</t>
+        </is>
+      </c>
+      <c r="B56" s="25" t="inlineStr">
+        <is>
+          <t>ecosystemmarketplace.com</t>
+        </is>
+      </c>
+      <c r="C56" s="17" t="inlineStr">
+        <is>
+          <t>Carbon credit prices and market trends</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Replace CICES with SEEA EA reference list throughout services materials
Changed classification label from "CICES category" to "SEEA EA
reference list" with section numbers (6.1 provisioning, 6.2 nursery,
6.3 carbon, 6.4 coastal protection, 6.5 sediment, 6.6 cultural).

Updated in: services-slides.md, services_account_template.xlsx,
example_completed_accounts.xlsx, printable Word docs, and print
notebook copies.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/s-s-event-bogor/sessions/day-2/clinic/examples/example_completed_accounts.xlsx
+++ b/s-s-event-bogor/sessions/day-2/clinic/examples/example_completed_accounts.xlsx
@@ -588,6 +588,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr"/>
       <c r="B4" s="3" t="inlineStr">
@@ -865,6 +866,7 @@
         <v>10000</v>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
@@ -917,6 +919,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -1086,9 +1089,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
@@ -1189,6 +1191,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
@@ -1247,6 +1250,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1390,6 +1394,7 @@
         <v>10000</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
@@ -1438,6 +1443,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1768,6 +1774,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
@@ -1820,6 +1827,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1828,8 +1836,8 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>CICES
-category</t>
+          <t>SEEA EA
+reference list</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1867,7 +1875,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Provisioning</t>
+          <t>6.1 (Provisioning)</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
@@ -1896,7 +1904,7 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>Provisioning</t>
+          <t>6.1 (Provisioning)</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
@@ -1921,7 +1929,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Regulating</t>
+          <t>6.3 (Regulating)</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
@@ -1948,7 +1956,7 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>Regulating</t>
+          <t>6.4 (Regulating)</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
@@ -1975,7 +1983,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Regulating</t>
+          <t>6.2 (Regulating)</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
@@ -2002,7 +2010,7 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Regulating</t>
+          <t>6.5 (Regulating)</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
@@ -2027,7 +2035,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Cultural</t>
+          <t>6.6 (Cultural)</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
@@ -2052,7 +2060,7 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>Cultural</t>
+          <t>6.6 (Cultural)</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
@@ -2077,7 +2085,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Cultural</t>
+          <t>6.6 (Cultural)</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -2102,7 +2110,7 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>Cultural</t>
+          <t>6.6 (Cultural)</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
@@ -2119,6 +2127,7 @@
         <v>4200</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
@@ -2164,6 +2173,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2460,6 +2470,7 @@
         <v>3686585</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
@@ -2517,6 +2528,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -2608,6 +2620,7 @@
         <v>0.079</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
@@ -2726,6 +2739,8 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
@@ -2964,6 +2979,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3122,6 +3138,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
@@ -3311,6 +3328,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
@@ -3446,6 +3464,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
         <is>
@@ -3546,6 +3565,7 @@
       </c>
       <c r="E28" s="25" t="inlineStr"/>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="23" t="inlineStr">
         <is>
@@ -3673,6 +3693,7 @@
       </c>
       <c r="E34" s="25" t="inlineStr"/>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="23" t="inlineStr">
         <is>
@@ -3769,6 +3790,7 @@
       </c>
       <c r="E39" s="25" t="inlineStr"/>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
         <is>
@@ -3823,6 +3845,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix remaining CICES references and improve PDF landscape scaling
CICES fixes:
- Replaced "CICES category" with "SEEA EA reference list" in
  generate_examples.py, generate_blank_tables.py, generate_filled_examples.py
- Regenerated all affected Word docs and Excel files
- No more CICES references anywhere in the event materials

PDF improvements:
- Regenerated all 16 HTML-to-PDF conversions with landscape scaling
  (CSS @page { size: landscape }) to prevent content being cut off
- Updated all print notebook copies

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/s-s-event-bogor/sessions/day-2/clinic/examples/example_completed_accounts.xlsx
+++ b/s-s-event-bogor/sessions/day-2/clinic/examples/example_completed_accounts.xlsx
@@ -588,7 +588,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr"/>
       <c r="B4" s="3" t="inlineStr">
@@ -866,7 +865,6 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
@@ -919,7 +917,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -1089,8 +1086,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
@@ -1191,7 +1189,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
@@ -1250,7 +1247,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1394,7 +1390,6 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
@@ -1443,7 +1438,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1774,7 +1768,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
@@ -1827,7 +1820,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1875,7 +1867,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>6.1 (Provisioning)</t>
+          <t>Provisioning (6.1)</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
@@ -1904,7 +1896,7 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>6.1 (Provisioning)</t>
+          <t>Provisioning (6.1)</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
@@ -1929,7 +1921,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>6.3 (Regulating)</t>
+          <t>Regulating</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
@@ -1956,7 +1948,7 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>6.4 (Regulating)</t>
+          <t>Regulating</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
@@ -1983,7 +1975,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>6.2 (Regulating)</t>
+          <t>Regulating</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
@@ -2010,7 +2002,7 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>6.5 (Regulating)</t>
+          <t>Regulating</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
@@ -2035,7 +2027,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>6.6 (Cultural)</t>
+          <t>Cultural (6.6)</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
@@ -2060,7 +2052,7 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>6.6 (Cultural)</t>
+          <t>Cultural (6.6)</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
@@ -2085,7 +2077,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>6.6 (Cultural)</t>
+          <t>Cultural (6.6)</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -2110,7 +2102,7 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>6.6 (Cultural)</t>
+          <t>Cultural (6.6)</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
@@ -2127,7 +2119,6 @@
         <v>4200</v>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
@@ -2173,7 +2164,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2470,7 +2460,6 @@
         <v>3686585</v>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
@@ -2528,7 +2517,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -2620,7 +2608,6 @@
         <v>0.079</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
@@ -2739,8 +2726,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
@@ -2979,7 +2964,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3138,7 +3122,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
@@ -3328,7 +3311,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
@@ -3464,7 +3446,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
         <is>
@@ -3565,7 +3546,6 @@
       </c>
       <c r="E28" s="25" t="inlineStr"/>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="23" t="inlineStr">
         <is>
@@ -3693,7 +3673,6 @@
       </c>
       <c r="E34" s="25" t="inlineStr"/>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="23" t="inlineStr">
         <is>
@@ -3790,7 +3769,6 @@
       </c>
       <c r="E39" s="25" t="inlineStr"/>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
         <is>
@@ -3845,7 +3823,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>

</xml_diff>